<commit_message>
Remove consent filtering from validation and related documentation
</commit_message>
<xml_diff>
--- a/docs/processmaker-input-template.xlsx
+++ b/docs/processmaker-input-template.xlsx
@@ -421,21 +421,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,55 +445,50 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>consent</t>
+          <t>airtime_phone</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>airtime_phone</t>
+          <t>network</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>network</t>
+          <t>submissiondate</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>submissiondate</t>
+          <t>today</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>today</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>project_name</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>project_name</t>
+          <t>Project_Activity</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Project_Activity</t>
+          <t>department</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>survey</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>survey</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>case_remark</t>
         </is>
@@ -508,53 +502,48 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>712345678</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>712345678</t>
+          <t>Safaricom</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Safaricom</t>
+          <t>8/25/2026 10:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>8/25/2026 10:00</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
           <t>25aug2026</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="F2" t="n">
         <v>150</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Test Project</t>
+          <t>g05|Testing</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>g05|Testing</t>
+          <t>Projects</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Projects</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
         <is>
           <t>C#37166 22505AA RESP AIRTIME-KSH150 d05</t>
         </is>
@@ -568,53 +557,48 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>798765432</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>798765432</t>
+          <t>Airtel</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Airtel</t>
+          <t>8/25/2026 11:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>8/25/2026 11:00</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
           <t>25aug2026</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="F3" t="n">
         <v>200</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Test Project</t>
+          <t>g05|Testing</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>g05|Testing</t>
+          <t>Projects</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Projects</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
         <is>
           <t>C#37167 22505AA RESP AIRTIME-KSH200 d05</t>
         </is>
@@ -628,60 +612,52 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>722334455</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>722334455</t>
+          <t>Telkom</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Telkom</t>
+          <t>8/25/2026 12:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8/25/2026 12:00</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
           <t>25aug2026</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="F4" t="n">
         <v>100</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Test Project</t>
+          <t>g05|Testing</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>g05|Testing</t>
+          <t>Projects</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Projects</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid consent" error="Consent must be &quot;Yes&quot; or &quot;No&quot;." type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid network" error="Network must exactly match one of the allowed values (case-sensitive)." type="list">
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid network" error="Network must exactly match one of the allowed values (case-sensitive)." type="list">
       <formula1>"Safaricom,Airtel,Airtel Postpaid,Telkom,Telkom Postpaid"</formula1>
     </dataValidation>
   </dataValidations>
@@ -695,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -729,43 +705,43 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>consent</t>
+          <t>airtime_phone</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Required. Must be exactly "Yes" (case-insensitive). Any other value excludes the row.</t>
+          <t>Required. Kenyan phone number. Digits only after cleanup; a leading 254 or 0 prefix is stripped (0 only if 9 digits would remain longer than 9); must resolve to exactly 9 digits. Example: 254712345678 or 0712345678 or 712345678 all normalize the same way.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>airtime_phone</t>
+          <t>network</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Required. Kenyan phone number. Digits only after cleanup; a leading 254 or 0 prefix is stripped (0 only if 9 digits would remain longer than 9); must resolve to exactly 9 digits. Example: 254712345678 or 0712345678 or 712345678 all normalize the same way.</t>
+          <t>Required, case-sensitive. Must be exactly one of: Safaricom, Airtel, Airtel Postpaid, Telkom, Telkom Postpaid. Any other value is a hard error.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>network</t>
+          <t>submissiondate</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Required, case-sensitive. Must be exactly one of: Safaricom, Airtel, Airtel Postpaid, Telkom, Telkom Postpaid. Any other value is a hard error.</t>
+          <t>Optional. Not validated by the formatter; informational only.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>submissiondate</t>
+          <t>today</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -777,55 +753,55 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>today</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Optional. Not validated by the formatter; informational only.</t>
+          <t>Required. A positive number (KES). Zero, negative, or non-numeric values are rejected. Amounts above KES 10,000 are allowed but flagged as a warning.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>project_name</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Required. A positive number (KES). Zero, negative, or non-numeric values are rejected. Amounts above KES 10,000 are allowed but flagged as a warning.</t>
+          <t>Optional. Used only as part of the legacy Remark fallback when case_remark is blank.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>project_name</t>
+          <t>Project_Activity</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Optional. Used only as part of the legacy Remark fallback when case_remark is blank.</t>
+          <t>Optional (note capitalization). Used only as part of the legacy Remark fallback when case_remark is blank.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Project_Activity</t>
+          <t>department</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Optional (note capitalization). Used only as part of the legacy Remark fallback when case_remark is blank.</t>
+          <t>Optional. Not validated by the formatter; informational only.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>survey</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -837,22 +813,10 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>survey</t>
+          <t>case_remark</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Optional. Not validated by the formatter; informational only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>case_remark</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Optional but recommended. Fixed format: 'C#&lt;case_number&gt; &lt;project_code&gt; RESP AIRTIME-KSH&lt;amount&gt; &lt;activity_code&gt;', e.g. 'C#37166 22505AA RESP AIRTIME-KSH29400 d05'. Reformatted automatically to 'Case #&lt;case_number&gt; | &lt;project_code&gt; | RESP | AIRTIME KSH &lt;amount&gt; | &lt;activity_code&gt;'. If left blank, the Remark falls back to '{project_name} - {Project_Activity}'. The embedded amount is cross-checked against the row's real amount column (mismatch is a soft warning only).</t>
         </is>

</xml_diff>

<commit_message>
Enhance unique_id handling and update related documentation
- Introduced resolve_unique_id function to standardize unique_id processing.
- Updated validation to warn on blank unique_id while preserving row inclusion.
- Adjusted output formatting to ensure unique_id is reflected as Account Name.
- Revised documentation for clarity on unique_id and case_remark usage.
- Ensured phone numbers are written as numbers in Excel output.
</commit_message>
<xml_diff>
--- a/docs/processmaker-input-template.xlsx
+++ b/docs/processmaker-input-template.xlsx
@@ -698,7 +698,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Optional. Any identifier; written verbatim to the output 'Account Name' column.</t>
+          <t>The row's Respondent ID, Staff ID, Case ID or Reso ID — written verbatim to the output 'Account Name' column, which is how the payment is identified in OpenFloat. A blank value is kept but warned about.</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Optional but recommended. Fixed format: 'C#&lt;case_number&gt; &lt;project_code&gt; RESP AIRTIME-KSH&lt;amount&gt; &lt;activity_code&gt;', e.g. 'C#37166 22505AA RESP AIRTIME-KSH29400 d05'. Reformatted automatically to 'Case #&lt;case_number&gt; | &lt;project_code&gt; | RESP | AIRTIME KSH &lt;amount&gt; | &lt;activity_code&gt;'. If left blank, the Remark falls back to '{project_name} - {Project_Activity}'. The embedded amount is cross-checked against the row's real amount column (mismatch is a soft warning only).</t>
+          <t>Optional but recommended. Fixed format: 'C#&lt;case_number&gt; &lt;project_code&gt; RESP AIRTIME-KSH&lt;amount&gt; &lt;activity_code&gt;', e.g. 'C#37166 22505AA RESP AIRTIME-KSH29400 d05'. Written to the output 'Remark' column in that same format (spacing normalized), which is how it comes back on the OpenFloat Transaction Statement. If left blank, the Remark falls back to '{project_name} - {Project_Activity}'. The embedded amount is cross-checked against the row's real amount column (mismatch is a soft warning only).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Enhance identifier column detection and handling
- Added support for specifying an identifier column via form data in the validate and transform endpoints.
- Implemented logic to detect the identifier column from uploaded files, prioritizing user-specified columns and falling back to detection when necessary.
- Updated the CaseRollup model to handle short-form case remarks without amounts, ensuring proper rollup functionality.
- Enhanced validation to provide warnings for missing or empty identifier columns, improving user feedback.
- Refactored normalizer functions to support flexible column naming and detection logic.
- Added comprehensive tests for identifier column detection, validation, and case remark handling to ensure robustness.
</commit_message>
<xml_diff>
--- a/docs/processmaker-input-template.xlsx
+++ b/docs/processmaker-input-template.xlsx
@@ -698,7 +698,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The row's Respondent ID, Staff ID, Case ID or Reso ID — written verbatim to the output 'Account Name' column, which is how the payment is identified in OpenFloat. A blank value is kept but warned about.</t>
+          <t>The row's identifier — written verbatim to the output 'Account Name' column, which is how the payment is identified in OpenFloat. Rename this column to suit the run: anything combining an identifier word (Staff, Respondent, Unique, Case, Reso, Beneficiary) with ID/Number/Ref is recognized automatically, e.g. 'Staff ID' or 'Respondent Ref'. A column whose name contains Name, Phone, Amount or Remark is never treated as the identifier. The app shows which column it picked and lets you change it. A blank value is kept but warned about.</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Optional but recommended. Fixed format: 'C#&lt;case_number&gt; &lt;project_code&gt; RESP AIRTIME-KSH&lt;amount&gt; &lt;activity_code&gt;', e.g. 'C#37166 22505AA RESP AIRTIME-KSH29400 d05'. Written to the output 'Remark' column in that same format (spacing normalized), which is how it comes back on the OpenFloat Transaction Statement. If left blank, the Remark falls back to '{project_name} - {Project_Activity}'. The embedded amount is cross-checked against the row's real amount column (mismatch is a soft warning only).</t>
+          <t>Optional but recommended. Either the full format 'C#&lt;case_number&gt; &lt;project_code&gt; RESP AIRTIME-KSH&lt;amount&gt; &lt;activity_code&gt;', e.g. 'C#37166 22505AA RESP AIRTIME-KSH29400 d05', or just the case number, e.g. 'C# 38305'. Written to the output 'Remark' column in the same form (spacing normalized), which is how it comes back on the OpenFloat Transaction Statement. The full format also lets the statement report total each case and compare it against what was actually disbursed. If left blank, the Remark falls back to '{project_name} - {Project_Activity}'. The embedded amount is cross-checked against the row's real amount column (mismatch is a soft warning only).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Enhance Remark Composition with Project Code Support
- Updated `_request_config` to accept `project_code` alongside `account_name_column`.
- Modified file validation and transformation functions to utilize the new `project_code` parameter.
- Introduced `build_remark` and `build_remark_context` functions to handle remark composition based on project codes.
- Added logic to ensure project codes from the file take precedence over configured codes.
- Implemented comprehensive tests for project code handling in remarks, ensuring correct warnings and behavior.
- Refactored existing functions to improve readability and maintainability, including renaming `resolve_unique_id` to `read_text_cell`.
- Added new tests to validate project code functionality and its integration with existing remark generation logic.
</commit_message>
<xml_diff>
--- a/docs/processmaker-input-template.xlsx
+++ b/docs/processmaker-input-template.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -435,6 +435,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,6 +494,11 @@
           <t>case_remark</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>project_code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -548,6 +554,11 @@
           <t>C#37166 22505AA RESP AIRTIME-KSH150 d05</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>22505AA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -603,6 +614,11 @@
           <t>C#37167 22505AA RESP AIRTIME-KSH200 d05</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>22505AA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -654,6 +670,7 @@
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -671,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -813,12 +830,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>project_code</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Optional. The project code used in the Remark's case reference, e.g. '22505AA'. Only needed when case_remark is short ('C# 38305'); leave it blank and the app will ask for one instead. No spaces — a code with a space cannot go in a case reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>case_remark</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Optional but recommended. Either the full format 'C#&lt;case_number&gt; &lt;project_code&gt; RESP AIRTIME-KSH&lt;amount&gt; &lt;activity_code&gt;', e.g. 'C#37166 22505AA RESP AIRTIME-KSH29400 d05', or just the case number, e.g. 'C# 38305'. Written to the output 'Remark' column in the same form (spacing normalized), which is how it comes back on the OpenFloat Transaction Statement. The full format also lets the statement report total each case and compare it against what was actually disbursed. If left blank, the Remark falls back to '{project_name} - {Project_Activity}'. The embedded amount is cross-checked against the row's real amount column (mismatch is a soft warning only).</t>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Optional but recommended. Either the full format 'C#&lt;case_number&gt; &lt;project_code&gt; RESP AIRTIME-KSH&lt;amount&gt; &lt;activity_code&gt;', e.g. 'C#37166 22505AA RESP AIRTIME-KSH29400 d05', or just the case number, e.g. 'C# 38305'. Written to the output 'Remark' column in the same form (spacing normalized), which is how it comes back on the OpenFloat Transaction Statement. A short reference is completed automatically into the full format using the project_code column (or the project code typed in the app), the code before the '|' in Project_Activity, and the total amount for that case across this file. The full format lets the statement report total each case and compare it against what was actually disbursed. If left blank, the Remark falls back to '{project_name} - {Project_Activity}'. The embedded amount is cross-checked against the case's total across this file (mismatch is a soft warning only).</t>
         </is>
       </c>
     </row>

</xml_diff>